<commit_message>
To do list updated
</commit_message>
<xml_diff>
--- a/Planning/toDoList.xlsx
+++ b/Planning/toDoList.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t>Todo lijstje:</t>
   </si>
@@ -40,9 +40,6 @@
     <t>??-5-2014</t>
   </si>
   <si>
-    <t>??-5-2015</t>
-  </si>
-  <si>
     <t>??-5-2016</t>
   </si>
   <si>
@@ -130,20 +127,26 @@
     <t>Inladen data versnellen</t>
   </si>
   <si>
-    <t>DONE</t>
-  </si>
-  <si>
-    <t>Verschillende dataset's inladen</t>
-  </si>
-  <si>
     <t>Afbeeldingen maken voor het laadscherm en icoon e.d.</t>
+  </si>
+  <si>
+    <t>Dat werkt al wel, alleen niet zoals gewenst dus REDO!</t>
+  </si>
+  <si>
+    <t>Kan niet</t>
+  </si>
+  <si>
+    <t>Verschillende dataset's inladen en de juiste afbeeldingen</t>
+  </si>
+  <si>
+    <t>Mathijs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,8 +169,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -192,6 +202,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="18">
     <border>
@@ -406,7 +422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -421,7 +437,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -429,7 +444,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
@@ -437,7 +451,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -759,123 +790,129 @@
       <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="B3" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="D3" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="20" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="15"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23" t="s">
+      <c r="E4" s="22"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="24"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21" t="s">
+      <c r="C5" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="D5" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="20"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="22"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="26" t="s">
+      <c r="C6" s="21"/>
+      <c r="D6" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="22"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="33"/>
+      <c r="B7" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="24"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23" t="s">
+      <c r="C7" s="21"/>
+      <c r="D7" s="31">
+        <v>41054</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="27"/>
+      <c r="B8" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24" t="s">
+      <c r="C8" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="24"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23" t="s">
+      <c r="E8" s="22"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="25"/>
+      <c r="B9" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="23"/>
+      <c r="D9" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="22"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="23"/>
-      <c r="D8" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="24"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="27"/>
-      <c r="B9" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="24" t="s">
+      <c r="C10" s="21"/>
+      <c r="D10" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="24"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="11"/>
+      <c r="E10" s="22"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
-      <c r="D11" s="11" t="s">
-        <v>12</v>
+      <c r="D11" s="32" t="s">
+        <v>11</v>
       </c>
       <c r="E11" s="11"/>
     </row>
@@ -883,8 +920,8 @@
       <c r="A12" s="12"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="11" t="s">
-        <v>13</v>
+      <c r="D12" s="32" t="s">
+        <v>12</v>
       </c>
       <c r="E12" s="11"/>
     </row>
@@ -892,8 +929,8 @@
       <c r="A13" s="12"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
-      <c r="D13" s="11" t="s">
-        <v>14</v>
+      <c r="D13" s="32" t="s">
+        <v>13</v>
       </c>
       <c r="E13" s="11"/>
     </row>
@@ -901,8 +938,8 @@
       <c r="A14" s="12"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="11" t="s">
-        <v>15</v>
+      <c r="D14" s="32" t="s">
+        <v>14</v>
       </c>
       <c r="E14" s="11"/>
     </row>
@@ -910,8 +947,8 @@
       <c r="A15" s="12"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
-      <c r="D15" s="11" t="s">
-        <v>16</v>
+      <c r="D15" s="32" t="s">
+        <v>15</v>
       </c>
       <c r="E15" s="11"/>
     </row>
@@ -919,8 +956,8 @@
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="11" t="s">
-        <v>17</v>
+      <c r="D16" s="32" t="s">
+        <v>16</v>
       </c>
       <c r="E16" s="11"/>
     </row>
@@ -928,8 +965,8 @@
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="11" t="s">
-        <v>18</v>
+      <c r="D17" s="32" t="s">
+        <v>17</v>
       </c>
       <c r="E17" s="11"/>
     </row>
@@ -937,8 +974,8 @@
       <c r="A18" s="12"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="11" t="s">
-        <v>19</v>
+      <c r="D18" s="32" t="s">
+        <v>18</v>
       </c>
       <c r="E18" s="11"/>
     </row>
@@ -946,8 +983,8 @@
       <c r="A19" s="12"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="11" t="s">
-        <v>20</v>
+      <c r="D19" s="32" t="s">
+        <v>19</v>
       </c>
       <c r="E19" s="11"/>
     </row>
@@ -955,8 +992,8 @@
       <c r="A20" s="12"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="11" t="s">
-        <v>21</v>
+      <c r="D20" s="32" t="s">
+        <v>20</v>
       </c>
       <c r="E20" s="11"/>
     </row>
@@ -964,8 +1001,8 @@
       <c r="A21" s="12"/>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
-      <c r="D21" s="11" t="s">
-        <v>22</v>
+      <c r="D21" s="32" t="s">
+        <v>21</v>
       </c>
       <c r="E21" s="11"/>
     </row>
@@ -973,8 +1010,8 @@
       <c r="A22" s="12"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="11" t="s">
-        <v>23</v>
+      <c r="D22" s="32" t="s">
+        <v>22</v>
       </c>
       <c r="E22" s="11"/>
     </row>
@@ -982,8 +1019,8 @@
       <c r="A23" s="12"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="11" t="s">
-        <v>24</v>
+      <c r="D23" s="32" t="s">
+        <v>23</v>
       </c>
       <c r="E23" s="11"/>
     </row>
@@ -991,8 +1028,8 @@
       <c r="A24" s="12"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="11" t="s">
-        <v>25</v>
+      <c r="D24" s="32" t="s">
+        <v>24</v>
       </c>
       <c r="E24" s="11"/>
     </row>
@@ -1000,8 +1037,8 @@
       <c r="A25" s="12"/>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="11" t="s">
-        <v>26</v>
+      <c r="D25" s="32" t="s">
+        <v>25</v>
       </c>
       <c r="E25" s="11"/>
     </row>
@@ -1009,8 +1046,8 @@
       <c r="A26" s="12"/>
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="11" t="s">
-        <v>27</v>
+      <c r="D26" s="32" t="s">
+        <v>26</v>
       </c>
       <c r="E26" s="11"/>
     </row>
@@ -1018,8 +1055,8 @@
       <c r="A27" s="12"/>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
-      <c r="D27" s="11" t="s">
-        <v>28</v>
+      <c r="D27" s="32" t="s">
+        <v>27</v>
       </c>
       <c r="E27" s="11"/>
     </row>

</xml_diff>